<commit_message>
chore(sample): update sample data with realistic noisy eval cases
</commit_message>
<xml_diff>
--- a/sample_data/sample_input.xlsx
+++ b/sample_data/sample_input.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -413,85 +413,93 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J3"/>
+  <dimension ref="A1:L3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Name of Supplier</t>
+          <t>Unnamed: 3</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>Supplier GST No</t>
+          <t>Vendor Name</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>Date of Document</t>
+          <t>Buyer GSTIN</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>Value Of Invoice</t>
+          <t>Doc Date</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>IGST Amt</t>
+          <t>Total Invoice Value</t>
         </is>
       </c>
       <c r="F1" t="inlineStr">
         <is>
+          <t>IGST Value</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
           <t>CGST Amt</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>SGST Amt</t>
-        </is>
-      </c>
       <c r="H1" t="inlineStr">
         <is>
-          <t>Cess Amt</t>
+          <t>SGST Amount</t>
         </is>
       </c>
       <c r="I1" t="inlineStr">
         <is>
-          <t>HSN Code</t>
+          <t>HSN/SAC</t>
         </is>
       </c>
       <c r="J1" t="inlineStr">
         <is>
-          <t>Doc No</t>
+          <t>Doc Num</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>Voucher Number</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
+        <is>
+          <t>ITC Eligible</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Vendor A</t>
-        </is>
-      </c>
+      <c r="A2" t="inlineStr"/>
       <c r="B2" t="inlineStr">
         <is>
-          <t>27AABCU9603R1ZX</t>
+          <t>TechCorp Solutions</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>2024-04-01</t>
-        </is>
-      </c>
-      <c r="D2" t="n">
-        <v>15000</v>
+          <t>29AAKCS3836BIZS</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>2024-04-10</t>
+        </is>
       </c>
       <c r="E2" t="n">
-        <v>2700</v>
+        <v>50000</v>
       </c>
       <c r="F2" t="n">
-        <v>0</v>
+        <v>9000</v>
       </c>
       <c r="G2" t="n">
         <v>0</v>
@@ -499,56 +507,70 @@
       <c r="H2" t="n">
         <v>0</v>
       </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>8471</t>
-        </is>
+      <c r="I2" t="n">
+        <v>9983</v>
       </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>INV-001</t>
+          <t>INV-2024-001</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>VCH-991</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>Y</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Vendor B</t>
-        </is>
-      </c>
+      <c r="A3" t="inlineStr"/>
       <c r="B3" t="inlineStr">
         <is>
-          <t>29AAKCS3836BIZS</t>
+          <t>Acme Industries</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>2024-04-05</t>
-        </is>
-      </c>
-      <c r="D3" t="n">
-        <v>42000</v>
+          <t>27AABCU9603R1ZX</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>2024-04-12</t>
+        </is>
       </c>
       <c r="E3" t="n">
-        <v>7560</v>
+        <v>120000</v>
       </c>
       <c r="F3" t="n">
         <v>0</v>
       </c>
       <c r="G3" t="n">
-        <v>0</v>
+        <v>10800</v>
       </c>
       <c r="H3" t="n">
-        <v>0</v>
-      </c>
-      <c r="I3" t="inlineStr">
-        <is>
-          <t>9403</t>
-        </is>
+        <v>10800</v>
+      </c>
+      <c r="I3" t="n">
+        <v>8471</v>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>INV-002</t>
+          <t>INV-2024-002</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>VCH-992</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>N</t>
         </is>
       </c>
     </row>

</xml_diff>